<commit_message>
added icon for exe file and some tidy up of code for pyinstaller
</commit_message>
<xml_diff>
--- a/sample_data/dummy_customer_data_cleaned.xlsx
+++ b/sample_data/dummy_customer_data_cleaned.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\redmo\PycharmProjects\customer-data-cleaner\sample_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8808904A-F1DE-4AEB-832C-9FDD3533F42D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36310A23-212F-47E3-85CD-8E3BE82713C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{E5110DD4-E069-4BF5-88E9-68582D53513D}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Cleaned Data" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Cleaned Data'!$A$1:$G$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Cleaned Data'!$A$1:$G$19</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="110">
   <si>
     <t>customer_id</t>
   </si>
@@ -191,189 +191,168 @@
     <t>N91 H4F2</t>
   </si>
   <si>
-    <t>CUST010</t>
-  </si>
-  <si>
-    <t>Ronan Gallagher</t>
-  </si>
-  <si>
-    <t>ronan.gallagher@example.com</t>
-  </si>
-  <si>
-    <t>089 100 2010</t>
-  </si>
-  <si>
-    <t>27 Atlantic Way</t>
-  </si>
-  <si>
-    <t>Sligo</t>
-  </si>
-  <si>
-    <t>F91 R2V8</t>
-  </si>
-  <si>
     <t>CUST011</t>
   </si>
   <si>
     <t>Maeve Brennan</t>
   </si>
   <si>
+    <t>083 100 2011</t>
+  </si>
+  <si>
+    <t>11 Birch Close</t>
+  </si>
+  <si>
+    <t>K78 D6P4</t>
+  </si>
+  <si>
+    <t>CUST012</t>
+  </si>
+  <si>
+    <t>Fionn O'Sullivan</t>
+  </si>
+  <si>
+    <t>fionn.osullivan@example.com</t>
+  </si>
+  <si>
+    <t>085 100 2012</t>
+  </si>
+  <si>
+    <t>6 Lakeside Walk</t>
+  </si>
+  <si>
+    <t>Kerry</t>
+  </si>
+  <si>
+    <t>V93 A7N5</t>
+  </si>
+  <si>
+    <t>Louth</t>
+  </si>
+  <si>
+    <t>CUST014</t>
+  </si>
+  <si>
+    <t>Shane Fitzpatrick</t>
+  </si>
+  <si>
+    <t>shane.fitzpatrick@example.com</t>
+  </si>
+  <si>
+    <t>087 100 2014</t>
+  </si>
+  <si>
+    <t>35 Castle Road</t>
+  </si>
+  <si>
+    <t>Kildare</t>
+  </si>
+  <si>
+    <t>W91 T8C2</t>
+  </si>
+  <si>
+    <t>CUST015</t>
+  </si>
+  <si>
+    <t>Gráinne Connolly</t>
+  </si>
+  <si>
+    <t>grainne.connolly@example.com</t>
+  </si>
+  <si>
+    <t>089 100 2015</t>
+  </si>
+  <si>
+    <t>8 Beechwood Rise</t>
+  </si>
+  <si>
+    <t>Clare</t>
+  </si>
+  <si>
+    <t>V95 P3H6</t>
+  </si>
+  <si>
+    <t>CUST017</t>
+  </si>
+  <si>
+    <t>Ciara Flynn</t>
+  </si>
+  <si>
+    <t>ciara.flynn@example.com</t>
+  </si>
+  <si>
+    <t>085 100 2017</t>
+  </si>
+  <si>
+    <t>24 Glenmore Park</t>
+  </si>
+  <si>
+    <t>Waterford</t>
+  </si>
+  <si>
+    <t>X91 D2R7</t>
+  </si>
+  <si>
+    <t>CUST019</t>
+  </si>
+  <si>
+    <t>Emer Quinn</t>
+  </si>
+  <si>
+    <t>emer.quinn@example.com</t>
+  </si>
+  <si>
+    <t>087 100 2019</t>
+  </si>
+  <si>
+    <t>29 Chapel Court</t>
+  </si>
+  <si>
+    <t>A92 C4N8</t>
+  </si>
+  <si>
+    <t>CUST003</t>
+  </si>
+  <si>
+    <t>Niamh Kelly</t>
+  </si>
+  <si>
+    <t>niamh.kelly@example.com</t>
+  </si>
+  <si>
+    <t>086 100 2003</t>
+  </si>
+  <si>
+    <t>22 Oakfield Park</t>
+  </si>
+  <si>
+    <t>D03 F8R4</t>
+  </si>
+  <si>
+    <t>CUST007</t>
+  </si>
+  <si>
+    <t>Orla Doyle</t>
+  </si>
+  <si>
+    <t>orla.doyle@example.com</t>
+  </si>
+  <si>
+    <t>085 100 2007</t>
+  </si>
+  <si>
+    <t>18 Riverbank Drive</t>
+  </si>
+  <si>
+    <t>Wicklow</t>
+  </si>
+  <si>
+    <t>A98 M3T6</t>
+  </si>
+  <si>
     <t>maeve.brennan@example.com</t>
   </si>
   <si>
-    <t>083 100 2011</t>
-  </si>
-  <si>
-    <t>11 Birch Close</t>
-  </si>
-  <si>
-    <t>K78 D6P4</t>
-  </si>
-  <si>
-    <t>CUST012</t>
-  </si>
-  <si>
-    <t>Fionn O'Sullivan</t>
-  </si>
-  <si>
-    <t>fionn.osullivan@example.com</t>
-  </si>
-  <si>
-    <t>085 100 2012</t>
-  </si>
-  <si>
-    <t>6 Lakeside Walk</t>
-  </si>
-  <si>
-    <t>Kerry</t>
-  </si>
-  <si>
-    <t>V93 A7N5</t>
-  </si>
-  <si>
-    <t>Louth</t>
-  </si>
-  <si>
-    <t>CUST014</t>
-  </si>
-  <si>
-    <t>Shane Fitzpatrick</t>
-  </si>
-  <si>
-    <t>shane.fitzpatrick@example.com</t>
-  </si>
-  <si>
-    <t>087 100 2014</t>
-  </si>
-  <si>
-    <t>35 Castle Road</t>
-  </si>
-  <si>
-    <t>Kildare</t>
-  </si>
-  <si>
-    <t>W91 T8C2</t>
-  </si>
-  <si>
-    <t>CUST015</t>
-  </si>
-  <si>
-    <t>Gráinne Connolly</t>
-  </si>
-  <si>
-    <t>grainne.connolly@example.com</t>
-  </si>
-  <si>
-    <t>089 100 2015</t>
-  </si>
-  <si>
-    <t>8 Beechwood Rise</t>
-  </si>
-  <si>
-    <t>Clare</t>
-  </si>
-  <si>
-    <t>V95 P3H6</t>
-  </si>
-  <si>
-    <t>CUST016</t>
-  </si>
-  <si>
-    <t>Padraig O'Neill</t>
-  </si>
-  <si>
-    <t>padraig.oneill@example.com</t>
-  </si>
-  <si>
-    <t>083 100 2016</t>
-  </si>
-  <si>
-    <t>16 Station View</t>
-  </si>
-  <si>
-    <t>N37 K9W4</t>
-  </si>
-  <si>
-    <t>CUST017</t>
-  </si>
-  <si>
-    <t>Ciara Flynn</t>
-  </si>
-  <si>
-    <t>ciara.flynn@example.com</t>
-  </si>
-  <si>
-    <t>085 100 2017</t>
-  </si>
-  <si>
-    <t>24 Glenmore Park</t>
-  </si>
-  <si>
-    <t>Waterford</t>
-  </si>
-  <si>
-    <t>X91 D2R7</t>
-  </si>
-  <si>
-    <t>CUST018</t>
-  </si>
-  <si>
-    <t>Oisín Murray</t>
-  </si>
-  <si>
-    <t>oisin.murray@example.com</t>
-  </si>
-  <si>
-    <t>086 100 2018</t>
-  </si>
-  <si>
-    <t>10 Orchard Green</t>
-  </si>
-  <si>
-    <t>Donegal</t>
-  </si>
-  <si>
-    <t>F92 Y6M3</t>
-  </si>
-  <si>
-    <t>CUST019</t>
-  </si>
-  <si>
-    <t>Emer Quinn</t>
-  </si>
-  <si>
-    <t>emer.quinn@example.com</t>
-  </si>
-  <si>
-    <t>087 100 2019</t>
-  </si>
-  <si>
-    <t>29 Chapel Court</t>
-  </si>
-  <si>
-    <t>A92 C4N8</t>
-  </si>
-  <si>
     <t>CUST020</t>
   </si>
   <si>
@@ -393,45 +372,6 @@
   </si>
   <si>
     <t>E91 V5F7</t>
-  </si>
-  <si>
-    <t>CUST003</t>
-  </si>
-  <si>
-    <t>Niamh Kelly</t>
-  </si>
-  <si>
-    <t>niamh.kelly@example.com</t>
-  </si>
-  <si>
-    <t>086 100 2003</t>
-  </si>
-  <si>
-    <t>22 Oakfield Park</t>
-  </si>
-  <si>
-    <t>D03 F8R4</t>
-  </si>
-  <si>
-    <t>CUST007</t>
-  </si>
-  <si>
-    <t>Orla Doyle</t>
-  </si>
-  <si>
-    <t>orla.doyle@example.com</t>
-  </si>
-  <si>
-    <t>085 100 2007</t>
-  </si>
-  <si>
-    <t>18 Riverbank Drive</t>
-  </si>
-  <si>
-    <t>Wicklow</t>
-  </si>
-  <si>
-    <t>A98 M3T6</t>
   </si>
 </sst>
 </file>
@@ -806,7 +746,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{54691E82-662D-4AC2-88E6-BFAED0AD7F5E}">
-  <dimension ref="A1:G21"/>
+  <sheetPr filterMode="1"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.81640625" bestFit="1" customWidth="1"/>
@@ -841,7 +782,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>7</v>
       </c>
@@ -864,7 +805,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>14</v>
       </c>
@@ -887,165 +828,165 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
-        <v>117</v>
+        <v>76</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>118</v>
+        <v>77</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>119</v>
+        <v>78</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>120</v>
+        <v>79</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>121</v>
+        <v>80</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>21</v>
+        <v>81</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B7" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C7" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="D7" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="E7" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="F7" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="G5" s="1" t="s">
+      <c r="G7" s="1" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A6" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A7" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
-        <v>123</v>
+        <v>83</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>124</v>
+        <v>84</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>125</v>
+        <v>85</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>126</v>
+        <v>86</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>127</v>
+        <v>87</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>128</v>
+        <v>61</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
-        <v>123</v>
+        <v>54</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>124</v>
+        <v>55</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>125</v>
+        <v>56</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>126</v>
+        <v>57</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>127</v>
+        <v>58</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>128</v>
+        <v>59</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
-        <v>42</v>
+        <v>69</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>43</v>
+        <v>70</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>44</v>
+        <v>71</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>45</v>
+        <v>72</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>46</v>
+        <v>73</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>47</v>
+        <v>74</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>48</v>
+        <v>75</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.35">
@@ -1056,253 +997,216 @@
         <v>50</v>
       </c>
       <c r="C11" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="D11" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="D11" s="1" t="s">
+      <c r="E11" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="E11" s="1" t="s">
+      <c r="F11" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G11" s="1" t="s">
         <v>53</v>
-      </c>
-      <c r="F11" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="G11" s="1" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>58</v>
+        <v>102</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="F12" s="1" t="s">
         <v>21</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
-        <v>62</v>
+        <v>89</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>63</v>
+        <v>90</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>64</v>
+        <v>91</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>65</v>
+        <v>92</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>66</v>
+        <v>93</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>67</v>
+        <v>21</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>68</v>
+        <v>94</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
-        <v>117</v>
+        <v>95</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>118</v>
+        <v>96</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>119</v>
+        <v>97</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>120</v>
+        <v>98</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>121</v>
+        <v>99</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>21</v>
+        <v>100</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>122</v>
+        <v>101</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
-        <v>70</v>
+        <v>95</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>71</v>
+        <v>96</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>72</v>
+        <v>97</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>73</v>
+        <v>98</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>74</v>
+        <v>99</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
-        <v>77</v>
+        <v>29</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>78</v>
+        <v>30</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>79</v>
+        <v>31</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>80</v>
+        <v>32</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>81</v>
+        <v>33</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>82</v>
+        <v>34</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
-        <v>84</v>
+        <v>62</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>85</v>
+        <v>63</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>86</v>
+        <v>64</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>87</v>
+        <v>65</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>88</v>
+        <v>66</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>47</v>
+        <v>67</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>89</v>
+        <v>68</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>91</v>
+        <v>104</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>92</v>
+        <v>105</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>93</v>
+        <v>106</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>94</v>
+        <v>107</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>95</v>
+        <v>108</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>96</v>
+        <v>109</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A20" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="E20" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="F20" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="G20" s="1" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A21" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="E21" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="F21" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="G21" s="1" t="s">
-        <v>116</v>
-      </c>
-    </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G21">
+  <autoFilter ref="A1:G19" xr:uid="{54691E82-662D-4AC2-88E6-BFAED0AD7F5E}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="CUST007"/>
+        <filter val="CUST011"/>
+        <filter val="CUST020"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G19">
     <sortCondition ref="B2"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>